<commit_message>
Update hardware BOM with XT30 cable item
</commit_message>
<xml_diff>
--- a/hardware/HEI_ReBot_Lift_BOM.xlsx
+++ b/hardware/HEI_ReBot_Lift_BOM.xlsx
@@ -1818,11 +1818,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W216"/>
+  <dimension ref="A1:W217"/>
   <sheetFormatPr defaultColWidth="12" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="12" style="1" customWidth="1"/>
@@ -1969,431 +1969,440 @@
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>22</v>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>XT30单头线</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>XT30U黄母V2版，18AWG（0.75平方）红黑线; 50cm</t>
+        </is>
       </c>
       <c r="D7" s="3">
         <v>4</v>
       </c>
       <c r="E7" s="3">
+        <v>9</v>
+      </c>
+      <c r="F7" s="3">
+        <v>36</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>https://e.tb.cn/h.84Y2Y6OhkDc8Qd8?tk=0uragDI49y7 CZ193 「络黎XT30单头线XT30U转接线充电线带线插头延长线硅胶线特软软线」</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="2"/>
+      <c r="B8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="3">
+        <v>4</v>
+      </c>
+      <c r="E8" s="3">
         <v>16</v>
       </c>
-      <c r="F7" s="3">
+      <c r="F8" s="3">
         <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="2" t="s">
+    <row r="9" spans="1:7">
+      <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D9" s="3">
         <v>1</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E9" s="3">
         <v>429</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F9" s="3">
         <f t="shared" si="0"/>
         <v>429</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G9" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
+    <row r="10" spans="1:7">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D10" s="3">
         <v>2</v>
       </c>
-      <c r="E9" s="3">
+      <c r="E10" s="3">
         <v>5</v>
       </c>
-      <c r="F9" s="3">
+      <c r="F10" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3" t="s">
+    <row r="11" spans="1:7">
+      <c r="A11" s="2"/>
+      <c r="B11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D11" s="3">
         <v>1</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E11" s="3">
         <v>350</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F11" s="3">
         <f t="shared" si="0"/>
         <v>350</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D11" s="3">
-        <v>2</v>
-      </c>
-      <c r="E11" s="3">
-        <v>6</v>
-      </c>
-      <c r="F11" s="3">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D12" s="3">
         <v>2</v>
       </c>
       <c r="E12" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F12" s="3">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D13" s="3">
         <v>2</v>
       </c>
       <c r="E13" s="3">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F13" s="3">
         <f t="shared" si="0"/>
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>43</v>
+      <c r="A14" s="2"/>
+      <c r="B14" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D14" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E14" s="3">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="F14" s="3">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2" t="s">
-        <v>46</v>
+      <c r="A15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D15" s="3">
         <v>1</v>
       </c>
       <c r="E15" s="3">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="F15" s="3">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D16" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E16" s="3">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F16" s="3">
         <f t="shared" si="0"/>
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D17" s="3">
         <v>4</v>
       </c>
       <c r="E17" s="3">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="F17" s="3">
         <f t="shared" si="0"/>
-        <v>260</v>
+        <v>40</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" s="2"/>
       <c r="B18" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D18" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18" s="3">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="F18" s="3">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>260</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:7">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
       <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="B19" s="2" t="s">
+        <v>55</v>
+      </c>
       <c r="C19" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D19" s="3">
         <v>1</v>
       </c>
       <c r="E19" s="3">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F19" s="3">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>59</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="2"/>
-      <c r="B20" s="2" t="s">
-        <v>60</v>
-      </c>
+      <c r="B20" s="2"/>
       <c r="C20" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D20" s="3">
         <v>1</v>
       </c>
       <c r="E20" s="3">
-        <v>88</v>
+        <v>18</v>
       </c>
       <c r="F20" s="3">
         <f t="shared" si="0"/>
-        <v>88</v>
+        <v>18</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="2"/>
       <c r="B21" s="2" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D21" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="3">
-        <v>12</v>
+        <v>88</v>
       </c>
       <c r="F21" s="3">
         <f t="shared" si="0"/>
-        <v>24</v>
+        <v>88</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="2"/>
-      <c r="B22" s="3" t="s">
-        <v>66</v>
+      <c r="B22" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D22" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E22" s="3">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="F22" s="3">
         <f t="shared" si="0"/>
-        <v>148</v>
+        <v>24</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1" spans="1:7">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" s="2"/>
       <c r="B23" s="3" t="s">
         <v>66</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D23" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E23" s="3">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="F23" s="3">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>148</v>
       </c>
       <c r="G23" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:7">
+    <row r="24" ht="18" customHeight="1" spans="1:7">
       <c r="A24" s="2"/>
-      <c r="B24" s="2" t="s">
-        <v>70</v>
+      <c r="B24" s="3" t="s">
+        <v>66</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D24" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" s="3">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="F24" s="3">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="2"/>
       <c r="B25" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D25" s="3">
         <v>1</v>
       </c>
       <c r="E25" s="3">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="F25" s="3">
         <f t="shared" si="0"/>
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1" spans="1:22">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>74</v>
@@ -2411,255 +2420,240 @@
       <c r="G26" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="H26" s="3"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="2"/>
-      <c r="S26" s="2"/>
-      <c r="T26" s="2"/>
-      <c r="U26" s="2"/>
-      <c r="V26" s="2"/>
-    </row>
-    <row r="27" spans="1:7">
+    </row>
+    <row r="27" ht="18" customHeight="1" spans="1:22">
       <c r="A27" s="2"/>
       <c r="B27" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D27" s="3">
         <v>1</v>
       </c>
       <c r="E27" s="3">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="F27" s="3">
         <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="G27" s="6" t="s">
-        <v>79</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
+      <c r="O27" s="2"/>
+      <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
+      <c r="R27" s="2"/>
+      <c r="S27" s="2"/>
+      <c r="T27" s="2"/>
+      <c r="U27" s="2"/>
+      <c r="V27" s="2"/>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="2"/>
       <c r="B28" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D28" s="3">
         <v>1</v>
       </c>
       <c r="E28" s="3">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F28" s="3">
         <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>82</v>
+        <v>6</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="2"/>
       <c r="B29" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D29" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="3">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F29" s="3">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D30" s="3">
         <v>2</v>
       </c>
       <c r="E30" s="3">
-        <v>46.5</v>
+        <v>6</v>
       </c>
       <c r="F30" s="3">
         <f t="shared" si="0"/>
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D31" s="3">
         <v>2</v>
       </c>
       <c r="E31" s="3">
-        <v>14</v>
+        <v>46.5</v>
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>93</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="2"/>
       <c r="B32" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D32" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="3">
-        <v>3799</v>
+        <v>14</v>
       </c>
       <c r="F32" s="3">
         <f t="shared" si="0"/>
-        <v>3799</v>
+        <v>28</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1" spans="1:7">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" s="2"/>
       <c r="B33" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D33" s="3">
         <v>1</v>
       </c>
       <c r="E33" s="3">
-        <v>28</v>
+        <v>3799</v>
       </c>
       <c r="F33" s="3">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>3799</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1" spans="1:7">
       <c r="A34" s="2"/>
       <c r="B34" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D34" s="3">
         <v>1</v>
       </c>
       <c r="E34" s="3">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F34" s="3">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1" spans="1:23">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" spans="1:7">
       <c r="A35" s="2"/>
-      <c r="B35" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>102</v>
+      <c r="B35" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>99</v>
       </c>
       <c r="D35" s="3">
         <v>1</v>
       </c>
       <c r="E35" s="3">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F35" s="3">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="G35" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="I35" s="3"/>
-      <c r="J35" s="3"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2"/>
-      <c r="P35" s="2"/>
-      <c r="Q35" s="2"/>
-      <c r="R35" s="2"/>
-      <c r="S35" s="2"/>
-      <c r="T35" s="2"/>
-      <c r="U35" s="2"/>
-      <c r="V35" s="2"/>
-      <c r="W35" s="2"/>
-    </row>
-    <row r="36" spans="1:23">
+        <v>20</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" spans="1:23">
       <c r="A36" s="2"/>
       <c r="B36" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D36" s="3">
         <v>1</v>
       </c>
       <c r="E36" s="3">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="F36" s="3">
         <f t="shared" si="0"/>
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="I36" s="3"/>
       <c r="J36" s="3"/>
@@ -2677,26 +2671,26 @@
       <c r="V36" s="2"/>
       <c r="W36" s="2"/>
     </row>
-    <row r="37" ht="18" customHeight="1" spans="1:23">
+    <row r="37" spans="1:23">
       <c r="A37" s="2"/>
       <c r="B37" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D37" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E37" s="3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="F37" s="3">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="I37" s="3"/>
       <c r="J37" s="3"/>
@@ -2717,23 +2711,23 @@
     <row r="38" ht="18" customHeight="1" spans="1:23">
       <c r="A38" s="2"/>
       <c r="B38" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D38" s="3">
         <v>2</v>
       </c>
       <c r="E38" s="3">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F38" s="3">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="I38" s="3"/>
       <c r="J38" s="3"/>
@@ -2754,23 +2748,23 @@
     <row r="39" ht="18" customHeight="1" spans="1:23">
       <c r="A39" s="2"/>
       <c r="B39" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D39" s="3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E39" s="3">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="F39" s="3">
         <f t="shared" si="0"/>
-        <v>110</v>
+        <v>34</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="I39" s="3"/>
       <c r="J39" s="3"/>
@@ -2791,23 +2785,23 @@
     <row r="40" ht="18" customHeight="1" spans="1:23">
       <c r="A40" s="2"/>
       <c r="B40" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D40" s="3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E40" s="3">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="F40" s="3">
         <f t="shared" si="0"/>
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="I40" s="3"/>
       <c r="J40" s="3"/>
@@ -2828,23 +2822,23 @@
     <row r="41" ht="18" customHeight="1" spans="1:23">
       <c r="A41" s="2"/>
       <c r="B41" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D41" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" s="3">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="F41" s="3">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="I41" s="3"/>
       <c r="J41" s="3"/>
@@ -2864,19 +2858,21 @@
     </row>
     <row r="42" ht="18" customHeight="1" spans="1:23">
       <c r="A42" s="2"/>
-      <c r="B42" s="3"/>
+      <c r="B42" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="C42" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D42" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E42" s="3">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="F42" s="3">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="G42" s="6" t="s">
         <v>121</v>
@@ -2899,24 +2895,22 @@
     </row>
     <row r="43" ht="18" customHeight="1" spans="1:23">
       <c r="A43" s="2"/>
-      <c r="B43" s="3" t="s">
-        <v>123</v>
-      </c>
+      <c r="B43" s="3"/>
       <c r="C43" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D43" s="3">
         <v>1</v>
       </c>
       <c r="E43" s="3">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="F43" s="3">
         <f t="shared" si="0"/>
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I43" s="3"/>
       <c r="J43" s="3"/>
@@ -2936,9 +2930,11 @@
     </row>
     <row r="44" ht="18" customHeight="1" spans="1:23">
       <c r="A44" s="2"/>
-      <c r="B44" s="3"/>
+      <c r="B44" s="3" t="s">
+        <v>123</v>
+      </c>
       <c r="C44" s="3" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D44" s="3">
         <v>1</v>
@@ -2971,24 +2967,22 @@
     </row>
     <row r="45" ht="18" customHeight="1" spans="1:23">
       <c r="A45" s="2"/>
-      <c r="B45" s="3" t="s">
-        <v>127</v>
-      </c>
+      <c r="B45" s="3"/>
       <c r="C45" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="D45" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F45" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="I45" s="3"/>
       <c r="J45" s="3"/>
@@ -3008,9 +3002,11 @@
     </row>
     <row r="46" ht="18" customHeight="1" spans="1:23">
       <c r="A46" s="2"/>
-      <c r="B46" s="3"/>
+      <c r="B46" s="3" t="s">
+        <v>127</v>
+      </c>
       <c r="C46" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D46" s="3">
         <v>2</v>
@@ -3042,27 +3038,23 @@
       <c r="W46" s="2"/>
     </row>
     <row r="47" ht="18" customHeight="1" spans="1:23">
-      <c r="A47" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>132</v>
-      </c>
+      <c r="A47" s="2"/>
+      <c r="B47" s="3"/>
       <c r="C47" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D47" s="3">
+        <v>2</v>
+      </c>
+      <c r="E47" s="3">
         <v>3</v>
-      </c>
-      <c r="E47" s="3">
-        <v>208</v>
       </c>
       <c r="F47" s="3">
         <f t="shared" si="0"/>
-        <v>624</v>
+        <v>6</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I47" s="3"/>
       <c r="J47" s="3"/>
@@ -3080,125 +3072,126 @@
       <c r="V47" s="2"/>
       <c r="W47" s="2"/>
     </row>
-    <row r="48" spans="1:7">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>136</v>
+    <row r="48" ht="18" customHeight="1" spans="1:23">
+      <c r="A48" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>133</v>
       </c>
       <c r="D48" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E48" s="3">
-        <v>2600</v>
+        <v>208</v>
       </c>
       <c r="F48" s="3">
         <f t="shared" si="0"/>
-        <v>2600</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1" spans="1:7">
+        <v>624</v>
+      </c>
+      <c r="G48" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" s="2"/>
+      <c r="Q48" s="2"/>
+      <c r="R48" s="2"/>
+      <c r="S48" s="2"/>
+      <c r="T48" s="2"/>
+      <c r="U48" s="2"/>
+      <c r="V48" s="2"/>
+      <c r="W48" s="2"/>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" s="2"/>
       <c r="B49" s="2" t="s">
-        <v>138</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>139</v>
+        <v>135</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>136</v>
       </c>
       <c r="D49" s="3">
         <v>1</v>
       </c>
       <c r="E49" s="3">
-        <v>180</v>
+        <v>2600</v>
       </c>
       <c r="F49" s="3">
         <f t="shared" si="0"/>
-        <v>180</v>
+        <v>2600</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1" spans="1:7">
       <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
+      <c r="B50" s="2" t="s">
+        <v>138</v>
+      </c>
       <c r="C50" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D50" s="3">
         <v>1</v>
       </c>
       <c r="E50" s="3">
-        <v>23</v>
+        <v>180</v>
       </c>
       <c r="F50" s="3">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>180</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1" spans="1:23">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1" spans="1:7">
       <c r="A51" s="2"/>
-      <c r="B51" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C51" s="3" t="s">
-        <v>144</v>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="D51" s="3">
         <v>1</v>
       </c>
       <c r="E51" s="3">
-        <v>486</v>
+        <v>23</v>
       </c>
       <c r="F51" s="3">
         <f t="shared" si="0"/>
-        <v>486</v>
+        <v>23</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="H51" s="3"/>
-      <c r="I51" s="2"/>
-      <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-      <c r="M51" s="2"/>
-      <c r="N51" s="2"/>
-      <c r="O51" s="2"/>
-      <c r="P51" s="2"/>
-      <c r="Q51" s="2"/>
-      <c r="R51" s="2"/>
-      <c r="S51" s="2"/>
-      <c r="T51" s="2"/>
-      <c r="U51" s="2"/>
-      <c r="V51" s="2"/>
-      <c r="W51" s="2"/>
+        <v>142</v>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:23">
       <c r="A52" s="2"/>
       <c r="B52" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D52" s="3">
         <v>1</v>
       </c>
       <c r="E52" s="3">
-        <v>53</v>
+        <v>486</v>
       </c>
       <c r="F52" s="3">
         <f t="shared" si="0"/>
-        <v>53</v>
+        <v>486</v>
       </c>
       <c r="G52" s="4" t="s">
         <v>145</v>
@@ -3220,35 +3213,53 @@
       <c r="V52" s="2"/>
       <c r="W52" s="2"/>
     </row>
-    <row r="53" spans="1:7">
-      <c r="A53" s="2" t="s">
+    <row r="53" ht="18" customHeight="1" spans="1:23">
+      <c r="A53" s="2"/>
+      <c r="B53" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D53" s="3">
+        <v>1</v>
+      </c>
+      <c r="E53" s="3">
+        <v>53</v>
+      </c>
+      <c r="F53" s="3">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="H53" s="3"/>
+      <c r="I53" s="2"/>
+      <c r="J53" s="2"/>
+      <c r="K53" s="2"/>
+      <c r="L53" s="2"/>
+      <c r="M53" s="2"/>
+      <c r="N53" s="2"/>
+      <c r="O53" s="2"/>
+      <c r="P53" s="2"/>
+      <c r="Q53" s="2"/>
+      <c r="R53" s="2"/>
+      <c r="S53" s="2"/>
+      <c r="T53" s="2"/>
+      <c r="U53" s="2"/>
+      <c r="V53" s="2"/>
+      <c r="W53" s="2"/>
+    </row>
+    <row r="54" spans="1:7">
+      <c r="A54" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B53" s="2" t="s">
+      <c r="B54" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C53" s="2" t="s">
+      <c r="C54" s="2" t="s">
         <v>150</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F53" s="3">
-        <v>300</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="54" spans="2:7">
-      <c r="B54" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="C54" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>151</v>
@@ -3257,78 +3268,85 @@
         <v>152</v>
       </c>
       <c r="F54" s="3">
+        <v>300</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7">
+      <c r="B55" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F55" s="3">
         <v>3500</v>
       </c>
-      <c r="G54" s="4" t="s">
+      <c r="G55" s="4" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1" spans="2:7">
-      <c r="B55" s="2" t="s">
+    <row r="56" ht="18" customHeight="1" spans="2:7">
+      <c r="B56" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C56" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="D55" s="3">
+      <c r="D56" s="3">
         <v>2</v>
       </c>
-      <c r="E55" s="3">
+      <c r="E56" s="3">
         <v>7500</v>
       </c>
-      <c r="F55" s="3">
+      <c r="F56" s="3">
         <v>15000</v>
       </c>
-      <c r="G55" s="4" t="s">
+      <c r="G56" s="4" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="56" ht="18" customHeight="1" spans="1:7">
-      <c r="A56" s="2" t="s">
+    <row r="57" ht="18" customHeight="1" spans="1:7">
+      <c r="A57" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="B56" s="2" t="s">
+      <c r="B57" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C56" s="2" t="s">
+      <c r="C57" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="D56" s="3">
+      <c r="D57" s="3">
         <v>1</v>
       </c>
-      <c r="E56" s="3" t="s">
+      <c r="E57" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="F56" s="3">
+      <c r="F57" s="3">
         <v>300</v>
       </c>
-      <c r="G56" s="2"/>
-    </row>
-    <row r="57" spans="1:7">
-      <c r="A57" s="2" t="s">
+      <c r="G57" s="2"/>
+    </row>
+    <row r="58" spans="1:7">
+      <c r="A58" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="B57" s="2" t="s">
+      <c r="B58" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="C58" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="D57" s="3">
+      <c r="D58" s="3">
         <v>40</v>
-      </c>
-      <c r="E57" s="3"/>
-      <c r="F57" s="3"/>
-      <c r="G57" s="2"/>
-    </row>
-    <row r="58" spans="1:7">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="D58" s="3">
-        <v>20</v>
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
@@ -3337,8 +3355,8 @@
     <row r="59" spans="1:7">
       <c r="A59" s="2"/>
       <c r="B59" s="2"/>
-      <c r="C59" s="3" t="s">
-        <v>167</v>
+      <c r="C59" s="2" t="s">
+        <v>166</v>
       </c>
       <c r="D59" s="3">
         <v>20</v>
@@ -3350,34 +3368,34 @@
     <row r="60" spans="1:7">
       <c r="A60" s="2"/>
       <c r="B60" s="2"/>
-      <c r="C60" s="2" t="s">
-        <v>168</v>
+      <c r="C60" s="3" t="s">
+        <v>167</v>
       </c>
       <c r="D60" s="3">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
       <c r="G60" s="2"/>
     </row>
-    <row r="61" ht="18" customHeight="1" spans="1:7">
+    <row r="61" spans="1:7">
       <c r="A61" s="2"/>
       <c r="B61" s="2"/>
-      <c r="C61" s="3" t="s">
-        <v>169</v>
+      <c r="C61" s="2" t="s">
+        <v>168</v>
       </c>
       <c r="D61" s="3">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3"/>
       <c r="G61" s="2"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" ht="18" customHeight="1" spans="1:7">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D62" s="3">
         <v>50</v>
@@ -3386,40 +3404,40 @@
       <c r="F62" s="3"/>
       <c r="G62" s="2"/>
     </row>
-    <row r="63" ht="18" customHeight="1" spans="1:7">
+    <row r="63" spans="1:7">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D63" s="3">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3"/>
       <c r="G63" s="2"/>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" ht="18" customHeight="1" spans="1:7">
       <c r="A64" s="2"/>
       <c r="B64" s="2"/>
-      <c r="C64" s="2" t="s">
-        <v>172</v>
+      <c r="C64" s="3" t="s">
+        <v>171</v>
       </c>
       <c r="D64" s="3">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3"/>
       <c r="G64" s="2"/>
     </row>
-    <row r="65" ht="18" customHeight="1" spans="1:7">
+    <row r="65" spans="1:7">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D65" s="3">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3"/>
@@ -3429,22 +3447,22 @@
       <c r="A66" s="2"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="D66" s="3"/>
+        <v>173</v>
+      </c>
+      <c r="D66" s="3">
+        <v>6</v>
+      </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3"/>
       <c r="G66" s="2"/>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" ht="18" customHeight="1" spans="1:7">
       <c r="A67" s="2"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="D67" s="3">
-        <v>24</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="D67" s="3"/>
       <c r="E67" s="3"/>
       <c r="F67" s="3"/>
       <c r="G67" s="2"/>
@@ -3452,8 +3470,8 @@
     <row r="68" spans="1:7">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
-      <c r="C68" s="3" t="s">
-        <v>176</v>
+      <c r="C68" s="2" t="s">
+        <v>175</v>
       </c>
       <c r="D68" s="3">
         <v>24</v>
@@ -3465,23 +3483,23 @@
     <row r="69" spans="1:7">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
-      <c r="C69" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="D69" s="3"/>
+      <c r="C69" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="D69" s="3">
+        <v>24</v>
+      </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3"/>
       <c r="G69" s="2"/>
     </row>
-    <row r="70" ht="18" customHeight="1" spans="1:7">
+    <row r="70" spans="1:7">
       <c r="A70" s="2"/>
       <c r="B70" s="2"/>
       <c r="C70" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="D70" s="3">
-        <v>2</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="D70" s="3"/>
       <c r="E70" s="3"/>
       <c r="F70" s="3"/>
       <c r="G70" s="2"/>
@@ -3490,7 +3508,7 @@
       <c r="A71" s="2"/>
       <c r="B71" s="2"/>
       <c r="C71" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D71" s="3">
         <v>2</v>
@@ -3499,14 +3517,14 @@
       <c r="F71" s="3"/>
       <c r="G71" s="2"/>
     </row>
-    <row r="72" spans="1:7">
+    <row r="72" ht="18" customHeight="1" spans="1:7">
       <c r="A72" s="2"/>
       <c r="B72" s="2"/>
-      <c r="C72" s="3" t="s">
-        <v>180</v>
+      <c r="C72" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="D72" s="3">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3"/>
@@ -3516,7 +3534,7 @@
       <c r="A73" s="2"/>
       <c r="B73" s="2"/>
       <c r="C73" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D73" s="3">
         <v>10</v>
@@ -3525,27 +3543,27 @@
       <c r="F73" s="3"/>
       <c r="G73" s="2"/>
     </row>
-    <row r="74" ht="18" customHeight="1" spans="1:7">
+    <row r="74" spans="1:7">
       <c r="A74" s="2"/>
       <c r="B74" s="2"/>
       <c r="C74" s="3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D74" s="3">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3"/>
       <c r="G74" s="2"/>
     </row>
-    <row r="75" spans="1:7">
+    <row r="75" ht="18" customHeight="1" spans="1:7">
       <c r="A75" s="2"/>
       <c r="B75" s="2"/>
-      <c r="C75" s="2" t="s">
-        <v>183</v>
+      <c r="C75" s="3" t="s">
+        <v>182</v>
       </c>
       <c r="D75" s="3">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3"/>
@@ -3555,10 +3573,10 @@
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D76" s="3">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3"/>
@@ -3566,35 +3584,38 @@
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="2"/>
-      <c r="B77" s="2" t="s">
-        <v>185</v>
-      </c>
+      <c r="B77" s="2"/>
       <c r="C77" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D77" s="3">
-        <v>12</v>
-      </c>
-      <c r="E77" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F77" s="3">
-        <v>300</v>
-      </c>
-      <c r="G77" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="2"/>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" s="2"/>
-      <c r="D78" s="3"/>
-      <c r="E78" s="3"/>
-      <c r="F78" s="3"/>
-      <c r="G78" s="2"/>
+      <c r="B78" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="D78" s="3">
+        <v>12</v>
+      </c>
+      <c r="E78" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F78" s="3">
+        <v>300</v>
+      </c>
+      <c r="G78" s="4"/>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" s="2"/>
-      <c r="B79" s="7" t="s">
-        <v>187</v>
-      </c>
       <c r="D79" s="3"/>
       <c r="E79" s="3"/>
       <c r="F79" s="3"/>
@@ -3602,6 +3623,9 @@
     </row>
     <row r="80" spans="1:7">
       <c r="A80" s="2"/>
+      <c r="B80" s="7" t="s">
+        <v>187</v>
+      </c>
       <c r="D80" s="3"/>
       <c r="E80" s="3"/>
       <c r="F80" s="3"/>
@@ -3617,20 +3641,20 @@
     <row r="82" spans="1:7">
       <c r="A82" s="2"/>
       <c r="D82" s="3"/>
-      <c r="E82" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="F82" s="3">
-        <f>SUM(F2:F81)</f>
-        <v>33510</v>
-      </c>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
       <c r="G82" s="2"/>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="2"/>
       <c r="D83" s="3"/>
-      <c r="E83" s="3"/>
-      <c r="F83" s="3"/>
+      <c r="E83" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="F83" s="3">
+        <f>SUM(F2:F81)</f>
+        <v>33510</v>
+      </c>
       <c r="G83" s="2"/>
     </row>
     <row r="84" spans="1:7">
@@ -3663,8 +3687,6 @@
     </row>
     <row r="88" spans="1:7">
       <c r="A88" s="2"/>
-      <c r="B88" s="2"/>
-      <c r="C88" s="2"/>
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3"/>
@@ -4821,6 +4843,15 @@
       <c r="E216" s="3"/>
       <c r="F216" s="3"/>
       <c r="G216" s="2"/>
+    </row>
+    <row r="217" spans="1:7">
+      <c r="A217" s="2"/>
+      <c r="B217" s="2"/>
+      <c r="C217" s="2"/>
+      <c r="D217" s="3"/>
+      <c r="E217" s="3"/>
+      <c r="F217" s="3"/>
+      <c r="G217" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -4838,60 +4869,60 @@
     <mergeCell ref="B57:B76"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="G55" r:id="rId1" display="https://detail.tmall.com/item.htm?abbucket=20&amp;id=1042412233386&amp;mi_id=0000rOoR2WLKwqKbn008PkZKlSmDRvaOBBbj8riX4AO3ZGI&amp;ns=1&amp;priceTId=2147848217855037942932874e0e40&amp;skuId=6065255360559&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%228f32413981eb717a5da405f9dafd6471%22%7D&amp;xxc=taobaoSearch"/>
-    <hyperlink ref="G54" r:id="rId2" display="https://www.jlc-bj.com" tooltip="https://www.jlc-bj.com"/>
-    <hyperlink ref="G53" r:id="rId3" display="https://gy2025.com" tooltip="https://gy2025.com"/>
-    <hyperlink ref="G52" r:id="rId4" display="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开" tooltip="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开"/>
-    <hyperlink ref="G51" r:id="rId4" display="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开" tooltip="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开"/>
-    <hyperlink ref="G50" r:id="rId5" display="https://e.tb.cn/h.84aoco7tFLIk6Tz?tk=dDc2gwNDrnP CZ057 「国标纯铜电源线三芯0.75平方1.5米开关电源交流输入线350W500专用」"/>
-    <hyperlink ref="G49" r:id="rId6" display="https://e.tb.cn/h.8eBX815GT1MNCDF?tk=GiXygwNENFK CZ001 「明伟LRS-1000W1200W800开关电源集中供电220V转24V48伏直流变压器」"/>
-    <hyperlink ref="G48" r:id="rId7" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d791726688046.12952e8d3UCi02&amp;id=791726688046&amp;mi_id=0000Z-2s3ZK1SUohSo6b93HwnwmjXSsQou5JCvSfHN5nluE"/>
-    <hyperlink ref="G47" r:id="rId8" display="https://e.tb.cn/h.RG8GR4TqjMhqLTS?tk=GMoTg9QZNuz CZ193 「1080p摄像头高清宽动态广角无畸变高帧率树莓派电脑安卓USB免驱」 点击链接直接打开 或者 淘宝搜索直接打开"/>
-    <hyperlink ref="G46" r:id="rId9" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d619626584933.c85e2e8dBZtwYj&amp;id=619626584933&amp;mi_id=0000eSxljDcWe975hiim-qcRtIjha_nScOicdoW_lJNB2Vk"/>
-    <hyperlink ref="G45" r:id="rId9" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d619626584933.c85e2e8dBZtwYj&amp;id=619626584933&amp;mi_id=0000eSxljDcWe975hiim-qcRtIjha_nScOicdoW_lJNB2Vk"/>
-    <hyperlink ref="G44" r:id="rId10" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d948071912183.29ae2e8dbIZE1m&amp;id=948071912183&amp;mi_id=0000Eg7HwfliiSjr_Jf9_Qgp_VhEfXh_BRmwJfGjoXjHj4g"/>
-    <hyperlink ref="G43" r:id="rId10" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d948071912183.29ae2e8dbIZE1m&amp;id=948071912183&amp;mi_id=0000Eg7HwfliiSjr_Jf9_Qgp_VhEfXh_BRmwJfGjoXjHj4g"/>
-    <hyperlink ref="G42" r:id="rId11" display="https://e.tb.cn/h.8fRlzfId1nzLsZd?tk=ydTXgwn1ing tG-#22&gt;lD 「接线端子接线神器电线快速连接器快接头多功能对接对插接头按压式」"/>
-    <hyperlink ref="G41" r:id="rId11" display="https://e.tb.cn/h.8fRlzfId1nzLsZd?tk=ydTXgwn1ing tG-#22&gt;lD 「接线端子接线神器电线快速连接器快接头多功能对接对插接头按压式」"/>
-    <hyperlink ref="G40" r:id="rId12" display="https://e.tb.cn/h.8VABxxxWJciux0u?tk=xy30gwNUZ7y HU006 「特软耐高温硅胶线镀锡铜电线软线18 24 30AWG五色盒装DIY航模导线」"/>
-    <hyperlink ref="G39" r:id="rId13" display="https://e.tb.cn/h.8fisJHajRTb0UAt?tk=Xl5YgwNfycZ MF937 「特软硅胶双并线 30-8AWG连接电线排线 耐高温硅胶红黑双并线」"/>
-    <hyperlink ref="G38" r:id="rId14" display="https://e.tb.cn/h.8eaN9FVYBnaXNZT?tk=3LlogwnOrHG HU287 「RJ45插座网口网络直通头圆型USB母座超6类机柜钣金连接器网线高清HDMI对接头TYPE-C面板固定接口转接头防尘」"/>
-    <hyperlink ref="G37" r:id="rId15" display="https://e.tb.cn/h.8fRyrkeIz7crwfB?tk=iZUzgwn9aed HU071 「DC099带线5.5*2.1/2.5mm母座焊接电源插座大电流金属公母头12V24V」"/>
-    <hyperlink ref="G36" r:id="rId16" display="https://e.tb.cn/h.RF4wcRUdIQGVrA0?tk=nWdng9QPT9x HU071 「带耳朵DC电源插座 双耳固定孔DC5.5x2.1/2.5mm充电口母座注塑带线」 点击链接直接打开 或者 淘宝搜索直接打开"/>
-    <hyperlink ref="G35" r:id="rId17" display="https://e.tb.cn/h.8eBCEHZfWQXdh0i?tk=5Li2gwnr1li HU591 「塑料尼龙钢制铝拖链坦克链条线槽桥式全封闭电缆高速静音工程机床」"/>
-    <hyperlink ref="G34" r:id="rId18" display="https://e.tb.cn/h.8fi0I8siTy4MSzV?tk=D4gLgwmOMKQ HU006 「亚博智能jetson转接器dp转hdmi线4K高清显示屏连接口orin nano/nx」"/>
-    <hyperlink ref="G33" r:id="rId19" display="https://e.tb.cn/h.83zni5yphOhVe7o?tk=oic5gwmkwo8 CZ057 「英伟达Jetson Orin Nano/Xavier NX亚克力外壳TX2开发板机箱SUPER」"/>
-    <hyperlink ref="G32" r:id="rId20" display="https://e.tb.cn/h.8eCF5n39KLI7qyH?tk=bi5Ggwmo19A CZ009 「Jetson Orin Nano Super 8G官方开发套件Orin Nano模组AI视觉识别」"/>
-    <hyperlink ref="G31" r:id="rId21" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d708365168245.fd582e8d8wqe4i&amp;id=708365168245&amp;mi_id=0000h-1UNUnw7XyWnSEDckaY8gHu_SFLF5qtjps2oEKDeC8"/>
-    <hyperlink ref="G30" r:id="rId22" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d828564042177.3b787484pvqwZK&amp;id=828564042177&amp;from=cart&amp;skuId=5726239234374&amp;mi_id=0000d7dk5wNPdIvOetkiMrpo9_1hCE0viQET1RXF00PGKvk&amp;upStreamPrice=4650"/>
-    <hyperlink ref="G29" r:id="rId23" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d547233352646.3b787484PE5cjQ&amp;id=547233352646&amp;from=cart&amp;skuId=4995699381661&amp;mi_id=0000iWnWwasu6QIhj6iyGq6OeaUGpR6YXUQH5pKs1RNQn2w&amp;upStreamPrice=600"/>
-    <hyperlink ref="G28" r:id="rId24" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d729212927080.fd582e8d8wqe4i&amp;id=729212927080&amp;mi_id=00000yfMwNsjGjjWlHl0lrrUnOQVkK-qyUVP0sGpHGEP33c"/>
-    <hyperlink ref="G27" r:id="rId25" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d41107441353.3b7874849hs38w&amp;id=41107441353&amp;from=cart&amp;skuId=3101315285673&amp;mi_id=0000GQ3QSpJzQKQTCdufrD8H5bOF3HlQVTr9DCxQ2dQ7peA&amp;upStreamPrice=528"/>
-    <hyperlink ref="G26" r:id="rId26" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d709235914675.350b74841Cvfbv&amp;id=709235914675&amp;from=cart&amp;skuId=5149779067604&amp;mi_id=0000vncj1LYsWztjyEPgSrUnGHUv8_qnU8g2QWIlTaNYDk8&amp;upStreamPrice=1310"/>
-    <hyperlink ref="G25" r:id="rId26" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d709235914675.350b74841Cvfbv&amp;id=709235914675&amp;from=cart&amp;skuId=5149779067604&amp;mi_id=0000vncj1LYsWztjyEPgSrUnGHUv8_qnU8g2QWIlTaNYDk8&amp;upStreamPrice=1310"/>
-    <hyperlink ref="G24" r:id="rId27" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d658648726917.3b787484dkMTN6&amp;id=658648726917&amp;from=cart&amp;skuId=4925834991211&amp;mi_id=0000p46vXzF4p1yOdIAjY4p1TiSTVuTaGjUdZp65MBIf1dg&amp;upStreamPrice=4210"/>
-    <hyperlink ref="G23" r:id="rId28" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d662780224557.29ae2e8dbIZE1m&amp;id=662780224557&amp;mi_id=0000V5eNt0NsKo8f6eIZV2l9oOWhmxzNHXYk1uWrB4Ytwq8"/>
-    <hyperlink ref="G22" r:id="rId28" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d662780224557.29ae2e8dbIZE1m&amp;id=662780224557&amp;mi_id=0000V5eNt0NsKo8f6eIZV2l9oOWhmxzNHXYk1uWrB4Ytwq8"/>
-    <hyperlink ref="G21" r:id="rId29" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d552349663785.fd582e8d8wqe4i&amp;id=552349663785&amp;mi_id=0000ctMWL1oEDZU35v4V_vc2THBXMeZ7eHmYKkTVuzsIgNM"/>
-    <hyperlink ref="G20" r:id="rId30" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d859985772657.12952e8d3UCi02&amp;id=859985772657&amp;mi_id=0000oH1CX8koZdrfbhevD2XbW0dwYZ8oGDmehEfrlIr-ESs"/>
-    <hyperlink ref="G19" r:id="rId31" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d728638915097.fd582e8d8wqe4i&amp;id=728638915097&amp;mi_id=0000mRJUcBlP2ceHn3sjqxeCSKMu60wx7jYFORjk_x82GuQ"/>
-    <hyperlink ref="G18" r:id="rId32" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d522031626999.1acf2e8d69gOKg&amp;id=522031626999&amp;mi_id=0000ifSp7nm4trbX5ToNGBSYSpnJj42nSRNwl66HsAqyeEc"/>
-    <hyperlink ref="G17" r:id="rId33" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d639679565187.12952e8d3UCi02&amp;id=639679565187&amp;mi_id=0000eY2CNWY7XPCpyLsgKfC1rD_yRgfLNB6NBNl6d1j3m80"/>
-    <hyperlink ref="G16" r:id="rId34" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d781570215534.12952e8d3UCi02&amp;id=781570215534&amp;mi_id=00008ASGBAWiF82kdjKTL_Sh4wHC2d7yrXi5YI1iWiwas8A"/>
-    <hyperlink ref="G15" r:id="rId35" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d524929127650.3b787484pJ0dyc&amp;id=524929127650&amp;from=cart&amp;skuId=3921830860539&amp;mi_id=00003GMNQrGd3wwdxIk63cNSsn67P84gj5wN9yXWso7Wmqs&amp;upStreamPrice=1700"/>
-    <hyperlink ref="G14" r:id="rId36" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d641646267315.285a2e8dI1AxzH&amp;id=641646267315&amp;mi_id=0000atOD0lhqvvfUibvb9RSchdwhLvm1SSKQISEXXiugFhM"/>
-    <hyperlink ref="G13" r:id="rId37" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d567240850944.fd582e8d8wqe4i&amp;id=567240850944&amp;mi_id=0000ru5aX1EAoZj2U9TDMIO_b-wJgBQY83ZD7UuQB9vxlc8"/>
-    <hyperlink ref="G12" r:id="rId38" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d627448619941.fd582e8d8wqe4i&amp;id=627448619941&amp;mi_id=0000D_YRp9hyjwEnWfdDvHKwaEUcZFvDx_qaLtl6X1OSJXY"/>
-    <hyperlink ref="G11" r:id="rId39" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d44863501262.285a2e8dI1AxzH&amp;id=44863501262&amp;mi_id=0000FmZot1FDA5sOrXNQlVOOl64J0rE5X5u7VNvcZwKy9O4"/>
-    <hyperlink ref="G10" r:id="rId40" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d994915794027.12952e8d3UCi02&amp;id=994915794027&amp;mi_id=0000Sw3xu_S1gSdzE4ko0hfy9g1dgqeNIznTdIix0h26Ac0"/>
-    <hyperlink ref="G9" r:id="rId41" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d615361930715.285a2e8dI1AxzH&amp;id=615361930715&amp;mi_id=000045b9GvP_G1Nvl8pHU0AiCB5N5CSHiTn29fTSbcO2FZ4"/>
-    <hyperlink ref="G8" r:id="rId42" display=" https://e.tb.cn/h.8exLaJE0rK9YDGT?tk=W1smgwOj0wZ CZ005 「含增票GX80双导轨直线滚珠丝杆滑台模组含57电机铝合金十字工作台」"/>
-    <hyperlink ref="G7" r:id="rId43" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d822600109037.fd582e8d8wqe4i&amp;id=822600109037&amp;mi_id=00007hCATsE-fjaGZ8iuJly2mG3dCd0e-HZ9mHtnrk30L28"/>
-    <hyperlink ref="G6" r:id="rId43" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d822600109037.fd582e8d8wqe4i&amp;id=822600109037&amp;mi_id=00007hCATsE-fjaGZ8iuJly2mG3dCd0e-HZ9mHtnrk30L28"/>
-    <hyperlink ref="G5" r:id="rId44" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d17388859879.12952e8d3UCi02&amp;id=17388859879&amp;mi_id=0000-NI_TuQvJ2b2nIACNXgrPK27w4vRn6oTAIErTrsRIbE"/>
-    <hyperlink ref="G4" r:id="rId45" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d815333472865.350b7484N9Fz4P&amp;id=815333472865&amp;from=cart&amp;skuId=5965481553149&amp;mi_id=0000BNbL09n5XFvjNRr6vtn96lMH4owOh3OKcx_hjjT7bqU&amp;upStreamPrice=59900"/>
-    <hyperlink ref="G3" r:id="rId46" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d724149127063.12952e8d3UCi02&amp;id=724149127063&amp;mi_id=0000vnuYMd_jgGg35p3t_RXK9a-WOaOUkgYuErlDbZIQLII"/>
-    <hyperlink ref="G2" r:id="rId47" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d692637585058.285a2e8dI1AxzH&amp;id=692637585058&amp;mi_id=0000WR0RZu1aRQt_jHBZuA8WJPCOpOg6Jw_U5JGTtFloJfQ"/>
+    <hyperlink ref="G55" ns1:id="rId1" display="https://detail.tmall.com/item.htm?abbucket=20&amp;id=1042412233386&amp;mi_id=0000rOoR2WLKwqKbn008PkZKlSmDRvaOBBbj8riX4AO3ZGI&amp;ns=1&amp;priceTId=2147848217855037942932874e0e40&amp;skuId=6065255360559&amp;spm=a21n57.1.hoverItem.2&amp;utparam=%7B%22aplus_abtest%22%3A%228f32413981eb717a5da405f9dafd6471%22%7D&amp;xxc=taobaoSearch"/>
+    <hyperlink ref="G54" ns1:id="rId2" display="https://www.jlc-bj.com" tooltip="https://www.jlc-bj.com"/>
+    <hyperlink ref="G53" ns1:id="rId3" display="https://gy2025.com" tooltip="https://gy2025.com"/>
+    <hyperlink ref="G52" ns1:id="rId4" display="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开" tooltip="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开"/>
+    <hyperlink ref="G51" ns1:id="rId4" display="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开" tooltip="https://e.tb.cn/h.RGjiAu6lB5a378z?tk=4wDhg9Qo9ce CZ057 「24V锂电池组6串18650大容量25.2伏电瓶监控灯可充电户外电源电机」 点击链接直接打开 或者 淘宝搜索直接打开"/>
+    <hyperlink ref="G50" ns1:id="rId5" display="https://e.tb.cn/h.84aoco7tFLIk6Tz?tk=dDc2gwNDrnP CZ057 「国标纯铜电源线三芯0.75平方1.5米开关电源交流输入线350W500专用」"/>
+    <hyperlink ref="G49" ns1:id="rId6" display="https://e.tb.cn/h.8eBX815GT1MNCDF?tk=GiXygwNENFK CZ001 「明伟LRS-1000W1200W800开关电源集中供电220V转24V48伏直流变压器」"/>
+    <hyperlink ref="G48" ns1:id="rId7" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d791726688046.12952e8d3UCi02&amp;id=791726688046&amp;mi_id=0000Z-2s3ZK1SUohSo6b93HwnwmjXSsQou5JCvSfHN5nluE"/>
+    <hyperlink ref="G47" ns1:id="rId8" display="https://e.tb.cn/h.RG8GR4TqjMhqLTS?tk=GMoTg9QZNuz CZ193 「1080p摄像头高清宽动态广角无畸变高帧率树莓派电脑安卓USB免驱」 点击链接直接打开 或者 淘宝搜索直接打开"/>
+    <hyperlink ref="G46" ns1:id="rId9" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d619626584933.c85e2e8dBZtwYj&amp;id=619626584933&amp;mi_id=0000eSxljDcWe975hiim-qcRtIjha_nScOicdoW_lJNB2Vk"/>
+    <hyperlink ref="G45" ns1:id="rId9" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d619626584933.c85e2e8dBZtwYj&amp;id=619626584933&amp;mi_id=0000eSxljDcWe975hiim-qcRtIjha_nScOicdoW_lJNB2Vk"/>
+    <hyperlink ref="G44" ns1:id="rId10" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d948071912183.29ae2e8dbIZE1m&amp;id=948071912183&amp;mi_id=0000Eg7HwfliiSjr_Jf9_Qgp_VhEfXh_BRmwJfGjoXjHj4g"/>
+    <hyperlink ref="G43" ns1:id="rId10" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d948071912183.29ae2e8dbIZE1m&amp;id=948071912183&amp;mi_id=0000Eg7HwfliiSjr_Jf9_Qgp_VhEfXh_BRmwJfGjoXjHj4g"/>
+    <hyperlink ref="G42" ns1:id="rId11" display="https://e.tb.cn/h.8fRlzfId1nzLsZd?tk=ydTXgwn1ing tG-#22&gt;lD 「接线端子接线神器电线快速连接器快接头多功能对接对插接头按压式」"/>
+    <hyperlink ref="G41" ns1:id="rId11" display="https://e.tb.cn/h.8fRlzfId1nzLsZd?tk=ydTXgwn1ing tG-#22&gt;lD 「接线端子接线神器电线快速连接器快接头多功能对接对插接头按压式」"/>
+    <hyperlink ref="G40" ns1:id="rId12" display="https://e.tb.cn/h.8VABxxxWJciux0u?tk=xy30gwNUZ7y HU006 「特软耐高温硅胶线镀锡铜电线软线18 24 30AWG五色盒装DIY航模导线」"/>
+    <hyperlink ref="G39" ns1:id="rId13" display="https://e.tb.cn/h.8fisJHajRTb0UAt?tk=Xl5YgwNfycZ MF937 「特软硅胶双并线 30-8AWG连接电线排线 耐高温硅胶红黑双并线」"/>
+    <hyperlink ref="G38" ns1:id="rId14" display="https://e.tb.cn/h.8eaN9FVYBnaXNZT?tk=3LlogwnOrHG HU287 「RJ45插座网口网络直通头圆型USB母座超6类机柜钣金连接器网线高清HDMI对接头TYPE-C面板固定接口转接头防尘」"/>
+    <hyperlink ref="G37" ns1:id="rId15" display="https://e.tb.cn/h.8fRyrkeIz7crwfB?tk=iZUzgwn9aed HU071 「DC099带线5.5*2.1/2.5mm母座焊接电源插座大电流金属公母头12V24V」"/>
+    <hyperlink ref="G36" ns1:id="rId16" display="https://e.tb.cn/h.RF4wcRUdIQGVrA0?tk=nWdng9QPT9x HU071 「带耳朵DC电源插座 双耳固定孔DC5.5x2.1/2.5mm充电口母座注塑带线」 点击链接直接打开 或者 淘宝搜索直接打开"/>
+    <hyperlink ref="G35" ns1:id="rId17" display="https://e.tb.cn/h.8eBCEHZfWQXdh0i?tk=5Li2gwnr1li HU591 「塑料尼龙钢制铝拖链坦克链条线槽桥式全封闭电缆高速静音工程机床」"/>
+    <hyperlink ref="G34" ns1:id="rId18" display="https://e.tb.cn/h.8fi0I8siTy4MSzV?tk=D4gLgwmOMKQ HU006 「亚博智能jetson转接器dp转hdmi线4K高清显示屏连接口orin nano/nx」"/>
+    <hyperlink ref="G33" ns1:id="rId19" display="https://e.tb.cn/h.83zni5yphOhVe7o?tk=oic5gwmkwo8 CZ057 「英伟达Jetson Orin Nano/Xavier NX亚克力外壳TX2开发板机箱SUPER」"/>
+    <hyperlink ref="G32" ns1:id="rId20" display="https://e.tb.cn/h.8eCF5n39KLI7qyH?tk=bi5Ggwmo19A CZ009 「Jetson Orin Nano Super 8G官方开发套件Orin Nano模组AI视觉识别」"/>
+    <hyperlink ref="G31" ns1:id="rId21" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d708365168245.fd582e8d8wqe4i&amp;id=708365168245&amp;mi_id=0000h-1UNUnw7XyWnSEDckaY8gHu_SFLF5qtjps2oEKDeC8"/>
+    <hyperlink ref="G30" ns1:id="rId22" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d828564042177.3b787484pvqwZK&amp;id=828564042177&amp;from=cart&amp;skuId=5726239234374&amp;mi_id=0000d7dk5wNPdIvOetkiMrpo9_1hCE0viQET1RXF00PGKvk&amp;upStreamPrice=4650"/>
+    <hyperlink ref="G29" ns1:id="rId23" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d547233352646.3b787484PE5cjQ&amp;id=547233352646&amp;from=cart&amp;skuId=4995699381661&amp;mi_id=0000iWnWwasu6QIhj6iyGq6OeaUGpR6YXUQH5pKs1RNQn2w&amp;upStreamPrice=600"/>
+    <hyperlink ref="G28" ns1:id="rId24" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d729212927080.fd582e8d8wqe4i&amp;id=729212927080&amp;mi_id=00000yfMwNsjGjjWlHl0lrrUnOQVkK-qyUVP0sGpHGEP33c"/>
+    <hyperlink ref="G27" ns1:id="rId25" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d41107441353.3b7874849hs38w&amp;id=41107441353&amp;from=cart&amp;skuId=3101315285673&amp;mi_id=0000GQ3QSpJzQKQTCdufrD8H5bOF3HlQVTr9DCxQ2dQ7peA&amp;upStreamPrice=528"/>
+    <hyperlink ref="G26" ns1:id="rId26" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d709235914675.350b74841Cvfbv&amp;id=709235914675&amp;from=cart&amp;skuId=5149779067604&amp;mi_id=0000vncj1LYsWztjyEPgSrUnGHUv8_qnU8g2QWIlTaNYDk8&amp;upStreamPrice=1310"/>
+    <hyperlink ref="G25" ns1:id="rId26" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d709235914675.350b74841Cvfbv&amp;id=709235914675&amp;from=cart&amp;skuId=5149779067604&amp;mi_id=0000vncj1LYsWztjyEPgSrUnGHUv8_qnU8g2QWIlTaNYDk8&amp;upStreamPrice=1310"/>
+    <hyperlink ref="G24" ns1:id="rId27" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d658648726917.3b787484dkMTN6&amp;id=658648726917&amp;from=cart&amp;skuId=4925834991211&amp;mi_id=0000p46vXzF4p1yOdIAjY4p1TiSTVuTaGjUdZp65MBIf1dg&amp;upStreamPrice=4210"/>
+    <hyperlink ref="G23" ns1:id="rId28" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d662780224557.29ae2e8dbIZE1m&amp;id=662780224557&amp;mi_id=0000V5eNt0NsKo8f6eIZV2l9oOWhmxzNHXYk1uWrB4Ytwq8"/>
+    <hyperlink ref="G22" ns1:id="rId28" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d662780224557.29ae2e8dbIZE1m&amp;id=662780224557&amp;mi_id=0000V5eNt0NsKo8f6eIZV2l9oOWhmxzNHXYk1uWrB4Ytwq8"/>
+    <hyperlink ref="G21" ns1:id="rId29" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d552349663785.fd582e8d8wqe4i&amp;id=552349663785&amp;mi_id=0000ctMWL1oEDZU35v4V_vc2THBXMeZ7eHmYKkTVuzsIgNM"/>
+    <hyperlink ref="G20" ns1:id="rId30" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d859985772657.12952e8d3UCi02&amp;id=859985772657&amp;mi_id=0000oH1CX8koZdrfbhevD2XbW0dwYZ8oGDmehEfrlIr-ESs"/>
+    <hyperlink ref="G19" ns1:id="rId31" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d728638915097.fd582e8d8wqe4i&amp;id=728638915097&amp;mi_id=0000mRJUcBlP2ceHn3sjqxeCSKMu60wx7jYFORjk_x82GuQ"/>
+    <hyperlink ref="G18" ns1:id="rId32" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d522031626999.1acf2e8d69gOKg&amp;id=522031626999&amp;mi_id=0000ifSp7nm4trbX5ToNGBSYSpnJj42nSRNwl66HsAqyeEc"/>
+    <hyperlink ref="G17" ns1:id="rId33" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d639679565187.12952e8d3UCi02&amp;id=639679565187&amp;mi_id=0000eY2CNWY7XPCpyLsgKfC1rD_yRgfLNB6NBNl6d1j3m80"/>
+    <hyperlink ref="G16" ns1:id="rId34" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d781570215534.12952e8d3UCi02&amp;id=781570215534&amp;mi_id=00008ASGBAWiF82kdjKTL_Sh4wHC2d7yrXi5YI1iWiwas8A"/>
+    <hyperlink ref="G15" ns1:id="rId35" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d524929127650.3b787484pJ0dyc&amp;id=524929127650&amp;from=cart&amp;skuId=3921830860539&amp;mi_id=00003GMNQrGd3wwdxIk63cNSsn67P84gj5wN9yXWso7Wmqs&amp;upStreamPrice=1700"/>
+    <hyperlink ref="G14" ns1:id="rId36" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d641646267315.285a2e8dI1AxzH&amp;id=641646267315&amp;mi_id=0000atOD0lhqvvfUibvb9RSchdwhLvm1SSKQISEXXiugFhM"/>
+    <hyperlink ref="G13" ns1:id="rId37" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d567240850944.fd582e8d8wqe4i&amp;id=567240850944&amp;mi_id=0000ru5aX1EAoZj2U9TDMIO_b-wJgBQY83ZD7UuQB9vxlc8"/>
+    <hyperlink ref="G12" ns1:id="rId38" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d627448619941.fd582e8d8wqe4i&amp;id=627448619941&amp;mi_id=0000D_YRp9hyjwEnWfdDvHKwaEUcZFvDx_qaLtl6X1OSJXY"/>
+    <hyperlink ref="G11" ns1:id="rId39" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d44863501262.285a2e8dI1AxzH&amp;id=44863501262&amp;mi_id=0000FmZot1FDA5sOrXNQlVOOl64J0rE5X5u7VNvcZwKy9O4"/>
+    <hyperlink ref="G10" ns1:id="rId40" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d994915794027.12952e8d3UCi02&amp;id=994915794027&amp;mi_id=0000Sw3xu_S1gSdzE4ko0hfy9g1dgqeNIznTdIix0h26Ac0"/>
+    <hyperlink ref="G9" ns1:id="rId41" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d615361930715.285a2e8dI1AxzH&amp;id=615361930715&amp;mi_id=000045b9GvP_G1Nvl8pHU0AiCB5N5CSHiTn29fTSbcO2FZ4"/>
+    <hyperlink ref="G8" ns1:id="rId42" display=" https://e.tb.cn/h.8exLaJE0rK9YDGT?tk=W1smgwOj0wZ CZ005 「含增票GX80双导轨直线滚珠丝杆滑台模组含57电机铝合金十字工作台」"/>
+    <hyperlink ref="G7" ns1:id="rId43" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d822600109037.fd582e8d8wqe4i&amp;id=822600109037&amp;mi_id=00007hCATsE-fjaGZ8iuJly2mG3dCd0e-HZ9mHtnrk30L28"/>
+    <hyperlink ref="G6" ns1:id="rId43" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d822600109037.fd582e8d8wqe4i&amp;id=822600109037&amp;mi_id=00007hCATsE-fjaGZ8iuJly2mG3dCd0e-HZ9mHtnrk30L28"/>
+    <hyperlink ref="G5" ns1:id="rId44" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d17388859879.12952e8d3UCi02&amp;id=17388859879&amp;mi_id=0000-NI_TuQvJ2b2nIACNXgrPK27w4vRn6oTAIErTrsRIbE"/>
+    <hyperlink ref="G4" ns1:id="rId45" display="https://item.taobao.com/item.htm?spm=a1z0d.6639537%2F202410.item.d815333472865.350b7484N9Fz4P&amp;id=815333472865&amp;from=cart&amp;skuId=5965481553149&amp;mi_id=0000BNbL09n5XFvjNRr6vtn96lMH4owOh3OKcx_hjjT7bqU&amp;upStreamPrice=59900"/>
+    <hyperlink ref="G3" ns1:id="rId46" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d724149127063.12952e8d3UCi02&amp;id=724149127063&amp;mi_id=0000vnuYMd_jgGg35p3t_RXK9a-WOaOUkgYuErlDbZIQLII"/>
+    <hyperlink ref="G2" ns1:id="rId47" display="https://item.taobao.com/item.htm?spm=tbpc.boughtlist.suborder_itempic.d692637585058.285a2e8dI1AxzH&amp;id=692637585058&amp;mi_id=0000WR0RZu1aRQt_jHBZuA8WJPCOpOg6Jw_U5JGTtFloJfQ"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>